<commit_message>
Contrast sideways and trending continuation states
</commit_message>
<xml_diff>
--- a/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
+++ b/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R9393d3ad8d3e4cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="R3ed91881d3204188"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="R2985a7850ba94151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R9cb67bf019874a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Re1859ee85865480b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="Re28d9385afad4e18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,6 +99,11 @@
         <x:fgColor rgb="FFECEFF2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EEF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -129,7 +134,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -228,6 +233,18 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -268,7 +285,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Candidate ID"/>
@@ -732,13 +749,13 @@
         <x:v>Positive completed returns may carry more positive forward dependence when the path is inefficient/sideways or movement capacity is low-to-moderate; efficient trending paths more often show gain exhaustion.</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>No trading rule. Descriptive comparison of the positive-prior branch across fixed prior/forward horizons and frozen ER20 / ATR% states.</x:v>
+        <x:v>No trading rule. Paired descriptive comparison of positive-prior correlations in causal ER20-sideways versus ER20-trending states across the frozen 15x15 daily horizon surface.</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
-        <x:v>TSLA shows a weak 5-10-session continuation ridge; the 129-instrument atlas shows broad positive gain-branch signs in ER20-sideways cells and negative signs in ER20-trending cells.</x:v>
+        <x:v>The paired equal-sector contrast is +0.048; 92.9% of 225 cells favor sideways, and all 11 sector surfaces have positive median contrasts.</x:v>
       </x:c>
       <x:c r="I6" s="22" t="str">
-        <x:v>Point estimates are small, windows overlap, TSLA motivated the lane, and no single representative rule or fresh replication has been frozen.</x:v>
+        <x:v>Point estimates remain small and overlapping; 16 cells break the pattern; the same 2018-2023 history discovered and evaluated the contrast; no next-open baseline exists.</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>DESCRIPTIVE_BEHAVIORAL_LEAD</x:v>
@@ -750,13 +767,13 @@
         <x:v>SEALED</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
-        <x:v>Choose one narrative-first representative comparison before any new calculation; then freeze timing, state, baseline, and failure rule.</x:v>
+        <x:v>Decide whether to freeze one representative horizon and a next-open baseline test, or preserve the contrast as context while opening the separately designed 30-minute lane.</x:v>
       </x:c>
       <x:c r="N6" s="22" t="str">
         <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
       </x:c>
       <x:c r="O6" s="22" t="str">
-        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_wide_atlas_full_vocabulary_20260827/</x:v>
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_state_contrast_20260828/</x:v>
       </x:c>
       <x:c r="P6" s="22" t="str">
         <x:v>current slice; see git history</x:v>
@@ -777,7 +794,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re47cdd9dcdd54765"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51f9d00d80d4e77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1114,6 +1131,41 @@
         <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_abnormal_volume_veto_20260828/</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="104" customHeight="1">
+      <x:c r="A11" s="47" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="B11" s="46" t="str">
+        <x:v>BEHAV-MOM-01</x:v>
+      </x:c>
+      <x:c r="C11" s="46" t="str">
+        <x:v>ER20 sideways-vs-trending paired contrast</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="str">
+        <x:v>129 instruments; 88-stock equal-sector core; positive-prior 15x15 surface</x:v>
+      </x:c>
+      <x:c r="E11" s="46" t="str">
+        <x:v>Is positive-prior continuation more pronounced in causal ER20-sideways than ER20-trending states?</x:v>
+      </x:c>
+      <x:c r="F11" s="46" t="str">
+        <x:v>Paired median contrast +0.048; 92.9% of cells favor sideways; all 11 sectors have positive median contrasts. Sixteen cells are exceptions.</x:v>
+      </x:c>
+      <x:c r="G11" s="46" t="str">
+        <x:v>DESCRIPTIVE_PAIRED_STATE_CONTRAST</x:v>
+      </x:c>
+      <x:c r="H11" s="46" t="str">
+        <x:v>The earlier state split became an explicit paired, sector-balanced contrast with visible exceptions.</x:v>
+      </x:c>
+      <x:c r="I11" s="46" t="str">
+        <x:v>No horizon, next-open rule, baseline, independent confirmation, or post-2023 outcome was opened.</x:v>
+      </x:c>
+      <x:c r="J11" s="46" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="K11" s="46" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_state_contrast_20260828/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -1121,7 +1173,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R907a65e5654f4582"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fbbb37579654292"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1297,7 +1349,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf28542e6d1534161"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b06e5fb8f94e41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Translate continuation lead into next-open rules
</commit_message>
<xml_diff>
--- a/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
+++ b/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R9cb67bf019874a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Re1859ee85865480b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="Re28d9385afad4e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R02265cd43cc74772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Ra475f483573a4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="R739ea3fccd994a16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +104,11 @@
         <x:fgColor rgb="FFE6EEF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EEF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -134,7 +139,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -245,6 +250,18 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -285,7 +302,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Candidate ID"/>
@@ -743,22 +760,22 @@
         <x:v>Own-asset return geometry</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
-        <x:v>Behavioral lead</x:v>
+        <x:v>Proto-strategy</x:v>
       </x:c>
       <x:c r="F6" s="22" t="str">
-        <x:v>Positive completed returns may carry more positive forward dependence when the path is inefficient/sideways or movement capacity is low-to-moderate; efficient trending paths more often show gain exhaustion.</x:v>
+        <x:v>A positive completed 20-session return inside a causal ER20-sideways state may precede executable continuation after the next open.</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>No trading rule. Paired descriptive comparison of positive-prior correlations in causal ER20-sideways versus ER20-trending states across the frozen 15x15 daily horizon surface.</x:v>
+        <x:v>At close t require R20 &gt; 0 and ER20 &lt; 0.30; enter open t+1; exit after 5, 10, or 20 held sessions; ignore overlapping signals; charge 10 bp round trip.</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
-        <x:v>The paired equal-sector contrast is +0.048; 92.9% of 225 cells favor sideways, and all 11 sector surfaces have positive median contrasts.</x:v>
+        <x:v>Raw net median-asset returns were +5, +23, and +66 bp at 5, 10, and 20 sessions. Only the 20-session sideways-minus-trending contrast was positive under both aggregation lenses (+38 bp equal-sector; +5 bp pooled).</x:v>
       </x:c>
       <x:c r="I6" s="22" t="str">
-        <x:v>Point estimates remain small and overlapping; 16 cells break the pattern; the same 2018-2023 history discovered and evaluated the contrast; no next-open baseline exists.</x:v>
+        <x:v>The rule trailed unconditional same-horizon drift by 16, 10, and 14 bp. R20 &gt; 0 also detracted versus sideways-only by 7, 9, and 14 bp; sector breadth was weak.</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
-        <x:v>DESCRIPTIVE_BEHAVIORAL_LEAD</x:v>
+        <x:v>TRAIN_NEXT_OPEN_HORIZON_COMPARISON_COMPLETE_STOP_BEFORE_SELECTION_OR_OOS</x:v>
       </x:c>
       <x:c r="K6" s="22" t="str">
         <x:v>2018-2023 descriptive evidence only</x:v>
@@ -767,13 +784,13 @@
         <x:v>SEALED</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
-        <x:v>Decide whether to freeze one representative horizon and a next-open baseline test, or preserve the contrast as context while opening the separately designed 30-minute lane.</x:v>
+        <x:v>Huddle before any new calculation. Decide whether the 20-session state contrast deserves a separately frozen mechanism test without the positive-R20 condition, or remains context only. Do not select a horizon or open OOS from this result.</x:v>
       </x:c>
       <x:c r="N6" s="22" t="str">
         <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
       </x:c>
       <x:c r="O6" s="22" t="str">
-        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_state_contrast_20260828/</x:v>
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_next_open_rule_20260829/</x:v>
       </x:c>
       <x:c r="P6" s="22" t="str">
         <x:v>current slice; see git history</x:v>
@@ -794,7 +811,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51f9d00d80d4e77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd73874e775cf4d27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1166,6 +1183,41 @@
         <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_state_contrast_20260828/</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="118" customHeight="1">
+      <x:c r="A12" s="53" t="n">
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="B12" s="52" t="str">
+        <x:v>BEHAV-MOM-01</x:v>
+      </x:c>
+      <x:c r="C12" s="52" t="str">
+        <x:v>Minimal next-open daily rule</x:v>
+      </x:c>
+      <x:c r="D12" s="52" t="str">
+        <x:v>129 visible instruments; 88-stock equal-sector core; 2018-2023 TRAIN; 5/10/20-session holds</x:v>
+      </x:c>
+      <x:c r="E12" s="52" t="str">
+        <x:v>Does positive R20 inside causal ER20-sideways translate into a next-open continuation rule that improves on matched controls and unconditional drift?</x:v>
+      </x:c>
+      <x:c r="F12" s="52" t="str">
+        <x:v>Raw net returns were positive at all holds, but excess versus drift was -16/-10/-14 bp. Only 20d beat trending under both aggregation lenses (+38/+5 bp); the positive-R20 condition underperformed sideways-only at every hold.</x:v>
+      </x:c>
+      <x:c r="G12" s="52" t="str">
+        <x:v>TRAIN_NEXT_OPEN_HORIZON_COMPARISON_COMPLETE_STOP_BEFORE_SELECTION_OR_OOS</x:v>
+      </x:c>
+      <x:c r="H12" s="52" t="str">
+        <x:v>The descriptive lead became an auditable open-to-open proto-rule with a visible clock, costs, overlap policy, matched controls, and sector-balanced readout.</x:v>
+      </x:c>
+      <x:c r="I12" s="52" t="str">
+        <x:v>No horizon was selected; thresholds were not tuned; portfolio replay, post-2023 OOS, and 30-minute data remain sealed.</x:v>
+      </x:c>
+      <x:c r="J12" s="52" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="K12" s="52" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_next_open_rule_20260829/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -1173,7 +1225,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fbbb37579654292"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96764b0de63b4dd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1349,7 +1401,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b06e5fb8f94e41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7f0a3846de49a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Attribute the 20-session continuation clue
</commit_message>
<xml_diff>
--- a/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
+++ b/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R02265cd43cc74772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Ra475f483573a4493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="R739ea3fccd994a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R1903e22c33514a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Rc303233cd3014a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="Re887e3870dac493d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +109,11 @@
         <x:fgColor rgb="FFE6EEF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EEF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -139,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -262,6 +267,18 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -302,7 +319,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Candidate ID"/>
@@ -763,19 +780,19 @@
         <x:v>Proto-strategy</x:v>
       </x:c>
       <x:c r="F6" s="22" t="str">
-        <x:v>A positive completed 20-session return inside a causal ER20-sideways state may precede executable continuation after the next open.</x:v>
+        <x:v>A completed 20-session return inside a causal ER20-sideways state may contain different executable behavior depending on whether the prior return is positive or negative.</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>At close t require R20 &gt; 0 and ER20 &lt; 0.30; enter open t+1; exit after 5, 10, or 20 held sessions; ignore overlapping signals; charge 10 bp round trip.</x:v>
+        <x:v>At close t classify ER20 &lt; 0.30 versus ER20 &gt;= 0.30 and R20 sign; enter open t+1; exit after 20 held sessions; ignore overlapping signals; charge 10 bp round trip.</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
-        <x:v>Raw net median-asset returns were +5, +23, and +66 bp at 5, 10, and 20 sessions. Only the 20-session sideways-minus-trending contrast was positive under both aggregation lenses (+38 bp equal-sector; +5 bp pooled).</x:v>
+        <x:v>The frozen 20-day attribution showed that only sideways negative-R20 cleared unconditional drift under both primary lenses: +5.8 bp equal-sector and +3.7 bp core event-pooled. Seven of eleven sector medians had positive excess.</x:v>
       </x:c>
       <x:c r="I6" s="22" t="str">
-        <x:v>The rule trailed unconditional same-horizon drift by 16, 10, and 14 bp. R20 &gt; 0 also detracted versus sideways-only by 7, 9, and 14 bp; sector breadth was weak.</x:v>
+        <x:v>The original continuation branch was falsified: sideways positive-R20 trailed negative-R20 by 15-19 bp and trailed drift. The 20-day horizon was data-informed in the same TRAIN sample; the surviving margin is modest and the average path separates late.</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
-        <x:v>TRAIN_NEXT_OPEN_HORIZON_COMPARISON_COMPLETE_STOP_BEFORE_SELECTION_OR_OOS</x:v>
+        <x:v>TRAIN_20D_SIGN_STATE_ATTRIBUTION_COMPLETE_STOP_BEFORE_RULE_OR_OOS</x:v>
       </x:c>
       <x:c r="K6" s="22" t="str">
         <x:v>2018-2023 descriptive evidence only</x:v>
@@ -784,13 +801,13 @@
         <x:v>SEALED</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
-        <x:v>Huddle before any new calculation. Decide whether the 20-session state contrast deserves a separately frozen mechanism test without the positive-R20 condition, or remains context only. Do not select a horizon or open OOS from this result.</x:v>
+        <x:v>Huddle before any new calculation. Keep the continuation formulation stopped. Decide whether the negative-prior sideways rebound deserves a separate predeclared candidate row and rule; do not repurpose this continuation row, tune the horizon, or open OOS yet.</x:v>
       </x:c>
       <x:c r="N6" s="22" t="str">
         <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
       </x:c>
       <x:c r="O6" s="22" t="str">
-        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_next_open_rule_20260829/</x:v>
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_20d_attribution_20260829/</x:v>
       </x:c>
       <x:c r="P6" s="22" t="str">
         <x:v>current slice; see git history</x:v>
@@ -811,7 +828,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd73874e775cf4d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de2c49818354e55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1218,6 +1235,41 @@
         <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_next_open_rule_20260829/</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="118" customHeight="1">
+      <x:c r="A13" s="59" t="n">
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="B13" s="58" t="str">
+        <x:v>BEHAV-MOM-01</x:v>
+      </x:c>
+      <x:c r="C13" s="58" t="str">
+        <x:v>20d sign/state mechanism attribution</x:v>
+      </x:c>
+      <x:c r="D13" s="58" t="str">
+        <x:v>129 visible instruments; 88-stock equal-sector core; 2018-2023 TRAIN; one frozen 20-session hold</x:v>
+      </x:c>
+      <x:c r="E13" s="58" t="str">
+        <x:v>Is the prior 20-day sideways-state result continuation, negative-prior rebound, a general sideways effect, or a relative morphology artifact?</x:v>
+      </x:c>
+      <x:c r="F13" s="58" t="str">
+        <x:v>Only sideways negative-R20 cleared drift under both primary lenses (+5.8/+3.7 bp). Positive-R20 trailed negative-R20 by 15-19 bp; 7/11 sector medians supported the negative branch.</x:v>
+      </x:c>
+      <x:c r="G13" s="58" t="str">
+        <x:v>TRAIN_20D_SIGN_STATE_ATTRIBUTION_COMPLETE_STOP_BEFORE_RULE_OR_OOS</x:v>
+      </x:c>
+      <x:c r="H13" s="58" t="str">
+        <x:v>The mechanism changed identity: the continuation interpretation was falsified and a modest, sector-broad rebound lead became visible.</x:v>
+      </x:c>
+      <x:c r="I13" s="58" t="str">
+        <x:v>No rebound rule was selected; the 20-day horizon was not retuned; post-2023 OOS, portfolio replay, and 30-minute data remain sealed.</x:v>
+      </x:c>
+      <x:c r="J13" s="58" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="K13" s="58" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_20d_attribution_20260829/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -1225,7 +1277,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96764b0de63b4dd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7de1fc1314ea48f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1401,7 +1453,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7f0a3846de49a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R769f3a1b38e946b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Open the sideways loss rebound baseline
</commit_message>
<xml_diff>
--- a/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
+++ b/operator_hypothesis_lab/registries/proto_strategy_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="R1903e22c33514a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Rc303233cd3014a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="Re887e3870dac493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proto Strategies" sheetId="1" r:id="Ra941d8a2d77f4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="R965d0f7f77ed4dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="3" r:id="R84bb86cd2e5c49d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,6 +114,16 @@
         <x:fgColor rgb="FFE6EEF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8EBC8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EEF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -144,7 +154,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -279,6 +289,30 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -295,7 +329,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProtoStrategyTable" displayName="ProtoStrategyTable" ref="A4:P6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProtoStrategyTable" displayName="ProtoStrategyTable" ref="A4:P7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nickname"/>
@@ -319,7 +353,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvidenceLogTable" displayName="EvidenceLogTable" ref="A4:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Candidate ID"/>
@@ -777,31 +811,31 @@
         <x:v>Own-asset return geometry</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
-        <x:v>Proto-strategy</x:v>
+        <x:v>Stopped</x:v>
       </x:c>
       <x:c r="F6" s="22" t="str">
-        <x:v>A completed 20-session return inside a causal ER20-sideways state may contain different executable behavior depending on whether the prior return is positive or negative.</x:v>
+        <x:v>A positive completed 20-session return inside causal ER20-sideways was hypothesized to precede executable continuation.</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>At close t classify ER20 &lt; 0.30 versus ER20 &gt;= 0.30 and R20 sign; enter open t+1; exit after 20 held sessions; ignore overlapping signals; charge 10 bp round trip.</x:v>
+        <x:v>The final mechanism attribution separated positive and negative R20 at the inherited 20-session horizon under the same next-open clock.</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
-        <x:v>The frozen 20-day attribution showed that only sideways negative-R20 cleared unconditional drift under both primary lenses: +5.8 bp equal-sector and +3.7 bp core event-pooled. Seven of eleven sector medians had positive excess.</x:v>
+        <x:v>Positive R20 trailed negative R20 by 15-19 bp. Only the negative-prior branch cleared drift under both primary lenses.</x:v>
       </x:c>
       <x:c r="I6" s="22" t="str">
-        <x:v>The original continuation branch was falsified: sideways positive-R20 trailed negative-R20 by 15-19 bp and trailed drift. The 20-day horizon was data-informed in the same TRAIN sample; the surviving margin is modest and the average path separates late.</x:v>
+        <x:v>The continuation sign was wrong; the 20-day horizon was data-informed in the same TRAIN sample. Rebound evidence belongs to a separate research identity.</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
-        <x:v>TRAIN_20D_SIGN_STATE_ATTRIBUTION_COMPLETE_STOP_BEFORE_RULE_OR_OOS</x:v>
+        <x:v>STOP_CONTINUATION_INTERPRETATION_AFTER_SIGN_ATTRIBUTION</x:v>
       </x:c>
       <x:c r="K6" s="22" t="str">
-        <x:v>2018-2023 descriptive evidence only</x:v>
+        <x:v>2018-2023 TRAIN only</x:v>
       </x:c>
       <x:c r="L6" s="22" t="str">
         <x:v>SEALED</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
-        <x:v>Huddle before any new calculation. Keep the continuation formulation stopped. Decide whether the negative-prior sideways rebound deserves a separate predeclared candidate row and rule; do not repurpose this continuation row, tune the horizon, or open OOS yet.</x:v>
+        <x:v>Set this line down. Do not rescue it by reversing the sign, changing ER20, selecting 20 days, or importing results from the separate rebound line.</x:v>
       </x:c>
       <x:c r="N6" s="22" t="str">
         <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
@@ -810,6 +844,56 @@
         <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_20d_attribution_20260829/</x:v>
       </x:c>
       <x:c r="P6" s="22" t="str">
+        <x:v>current slice; see git history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="138" customHeight="1">
+      <x:c r="A7" s="64" t="str">
+        <x:v>BEHAV-MR-02</x:v>
+      </x:c>
+      <x:c r="B7" s="64" t="str">
+        <x:v>Sideways Loss Rebound</x:v>
+      </x:c>
+      <x:c r="C7" s="64" t="str">
+        <x:v>Mean reversion</x:v>
+      </x:c>
+      <x:c r="D7" s="64" t="str">
+        <x:v>Own-asset return geometry</x:v>
+      </x:c>
+      <x:c r="E7" s="64" t="str">
+        <x:v>Behavioral lead</x:v>
+      </x:c>
+      <x:c r="F7" s="64" t="str">
+        <x:v>After a negative completed 20-session return, an inefficient sideways path may identify a better rebound environment than negative return alone.</x:v>
+      </x:c>
+      <x:c r="G7" s="64" t="str">
+        <x:v>At close t require R20 &lt; 0 and ER20 &lt; 0.30; enter open t+1; exit after 20 held sessions; ignore overlap; charge 10 bp. Compare with negative-only, trending-negative, sideways-only, and drift.</x:v>
+      </x:c>
+      <x:c r="H7" s="64" t="str">
+        <x:v>Primary excess was +5.8 bp equal-sector and +3.7 bp pooled with 7/11 positive sectors, but incremental lift versus negative-only disagreed by weighting lens (-5.6/+4.3 bp).</x:v>
+      </x:c>
+      <x:c r="I7" s="64" t="str">
+        <x:v>Only 2/6 TRAIN years had positive primary excess. The ER20-sideways gate did not robustly improve on negative R20 alone; horizon and cutoff are data-informed.</x:v>
+      </x:c>
+      <x:c r="J7" s="64" t="str">
+        <x:v>TRAIN_SIDEWAYS_LOSS_REBOUND_BASELINE_COMPLETE_STOP_BEFORE_RULE_OR_OOS</x:v>
+      </x:c>
+      <x:c r="K7" s="64" t="str">
+        <x:v>2018-2023 TRAIN only</x:v>
+      </x:c>
+      <x:c r="L7" s="64" t="str">
+        <x:v>SEALED</x:v>
+      </x:c>
+      <x:c r="M7" s="64" t="str">
+        <x:v>Huddle before any new calculation. Do not add severity, tune ER20 or the 20-day horizon, select sectors or years, or open post-2023 OOS.</x:v>
+      </x:c>
+      <x:c r="N7" s="64" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_SIDEWAYS_LOSS_REBOUND_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="O7" s="64" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_sideways_loss_rebound_baseline_20260829/</x:v>
+      </x:c>
+      <x:c r="P7" s="64" t="str">
         <x:v>current slice; see git history</x:v>
       </x:c>
     </x:row>
@@ -828,7 +912,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de2c49818354e55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8702ab2316f44f34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1270,6 +1354,76 @@
         <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_20d_attribution_20260829/</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="118" customHeight="1">
+      <x:c r="A14" s="70" t="n">
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="B14" s="69" t="str">
+        <x:v>BEHAV-MOM-01</x:v>
+      </x:c>
+      <x:c r="C14" s="69" t="str">
+        <x:v>Continuation line closure</x:v>
+      </x:c>
+      <x:c r="D14" s="69" t="str">
+        <x:v>2018-2023 TRAIN; inherited 20-session attribution</x:v>
+      </x:c>
+      <x:c r="E14" s="69" t="str">
+        <x:v>Should the negative-prior result be used to reverse or rescue the continuation hypothesis?</x:v>
+      </x:c>
+      <x:c r="F14" s="69" t="str">
+        <x:v>No. Positive R20 was the wrong sign; the continuation interpretation is stopped and the rebound observation receives a separate identity.</x:v>
+      </x:c>
+      <x:c r="G14" s="69" t="str">
+        <x:v>STOP_CONTINUATION_INTERPRETATION_AFTER_SIGN_ATTRIBUTION</x:v>
+      </x:c>
+      <x:c r="H14" s="69" t="str">
+        <x:v>The hypothesis ledger now preserves a clean conceptual boundary between continuation and mean reversion.</x:v>
+      </x:c>
+      <x:c r="I14" s="69" t="str">
+        <x:v>No sign reversal, rule rescue, horizon selection, or OOS authority was granted.</x:v>
+      </x:c>
+      <x:c r="J14" s="69" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_DAILY_CONTINUATION_MICROSCOPE_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="K14" s="69" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_continuation_20d_attribution_20260829/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="118" customHeight="1">
+      <x:c r="A15" s="71" t="n">
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>BEHAV-MR-02</x:v>
+      </x:c>
+      <x:c r="C15" s="64" t="str">
+        <x:v>Sideways-loss matched-control baseline</x:v>
+      </x:c>
+      <x:c r="D15" s="64" t="str">
+        <x:v>129 visible instruments; 88-stock equal-sector core; 2018-2023 TRAIN; frozen 20-session hold</x:v>
+      </x:c>
+      <x:c r="E15" s="64" t="str">
+        <x:v>Does R20 &lt; 0 inside ER20-sideways add rebound discrimination beyond negative-only, trending-negative, sideways-only, and drift?</x:v>
+      </x:c>
+      <x:c r="F15" s="64" t="str">
+        <x:v>Primary excess was +5.8/+3.7 bp, but primary minus negative-only was -5.6 bp equal-sector and +4.3 bp pooled. Only 2/6 TRAIN years were positive-excess.</x:v>
+      </x:c>
+      <x:c r="G15" s="64" t="str">
+        <x:v>TRAIN_SIDEWAYS_LOSS_REBOUND_BASELINE_COMPLETE_STOP_BEFORE_RULE_OR_OOS</x:v>
+      </x:c>
+      <x:c r="H15" s="64" t="str">
+        <x:v>A distinct rebound identity and its first matched-control failure mode are now auditable.</x:v>
+      </x:c>
+      <x:c r="I15" s="64" t="str">
+        <x:v>No rule, severity gate, state/horizon tuning, sector/year selection, portfolio replay, or post-2023 OOS was opened.</x:v>
+      </x:c>
+      <x:c r="J15" s="64" t="str">
+        <x:v>operator_hypothesis_lab/docs/RETURN_GEOMETRY_SIDEWAYS_LOSS_REBOUND_2018_2023.md</x:v>
+      </x:c>
+      <x:c r="K15" s="64" t="str">
+        <x:v>runs/research_workbench/operator_hypothesis_lab/return_geometry_sideways_loss_rebound_baseline_20260829/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -1277,7 +1431,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7de1fc1314ea48f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c6f8aedd548400b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1453,7 +1607,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R769f3a1b38e946b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c4b537d7534d81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>